<commit_message>
Refactored nnTrainer to try to reduce memory consumption - because using 1d LSTM with 100 second window used over 100GB of RAM+swap!
</commit_message>
<xml_diff>
--- a/user_tools/nnTraining2/reports/cnn_lstm_sep2026/cnn_lstm_results_analysis.xlsx
+++ b/user_tools/nnTraining2/reports/cnn_lstm_sep2026/cnn_lstm_results_analysis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="41">
   <si>
     <t xml:space="preserve">Augmentation Effects Analysis</t>
   </si>
@@ -112,6 +112,12 @@
     <t xml:space="preserve">n/a</t>
   </si>
   <si>
+    <t xml:space="preserve">lstm_1d/14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise + User + SR (14)</t>
+  </si>
+  <si>
     <t xml:space="preserve">lstm_1d/12</t>
   </si>
   <si>
@@ -122,6 +128,18 @@
   </si>
   <si>
     <t xml:space="preserve">Noise + User + OS + SR + NS (13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lstm_1d/15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise + User + SR + 45sec (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lstm_1d/16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise + User + SR + 60sec (16)</t>
   </si>
   <si>
     <t xml:space="preserve">OSD</t>
@@ -165,6 +183,7 @@
     </font>
     <font>
       <sz val="13"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -176,6 +195,7 @@
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -359,8 +379,12 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB" sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Effect of Data Augmentation on ML Seizure Detection Model</a:t>
             </a:r>
@@ -446,7 +470,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$5:$B$18</c:f>
+              <c:f>Sheet1!$B$5:$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
@@ -474,16 +498,16 @@
                   <c:v>Noise + User (7)</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Noise + User + OS (8)</c:v>
+                  <c:v>Noise + User + NS (9)</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Noise + User + NS (9)</c:v>
+                  <c:v>Noise + User + SR (14)</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Noise + User + OS + SR (12)</c:v>
+                  <c:v>Noise + User + SR + 45sec (15)</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Noise + User + OS + SR + NS (13)</c:v>
+                  <c:v>Noise + User + SR + 60sec (16)</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>OSD</c:v>
@@ -493,7 +517,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$18</c:f>
+              <c:f>Sheet1!$E$5:$E$21</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -522,16 +546,16 @@
                   <c:v>0.51</c:v>
                 </c:pt>
                 <c:pt idx="8">
+                  <c:v>0.49</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>0.53</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.49</c:v>
-                </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.57</c:v>
+                  <c:v>0.63</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.55</c:v>
+                  <c:v>0.44</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0.46</c:v>
@@ -605,7 +629,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$5:$B$18</c:f>
+              <c:f>Sheet1!$B$5:$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
@@ -633,16 +657,16 @@
                   <c:v>Noise + User (7)</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Noise + User + OS (8)</c:v>
+                  <c:v>Noise + User + NS (9)</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Noise + User + NS (9)</c:v>
+                  <c:v>Noise + User + SR (14)</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Noise + User + OS + SR (12)</c:v>
+                  <c:v>Noise + User + SR + 45sec (15)</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Noise + User + OS + SR + NS (13)</c:v>
+                  <c:v>Noise + User + SR + 60sec (16)</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>OSD</c:v>
@@ -652,7 +676,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$5:$H$18</c:f>
+              <c:f>Sheet1!$H$5:$H$21</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -681,16 +705,13 @@
                   <c:v>0.49</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.53</c:v>
+                  <c:v>0.48</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.48</c:v>
+                  <c:v>0.62</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.65</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.64</c:v>
+                  <c:v>0.61</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0.46</c:v>
@@ -701,11 +722,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="72898365"/>
-        <c:axId val="80180890"/>
+        <c:axId val="96179303"/>
+        <c:axId val="31763613"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="72898365"/>
+        <c:axId val="96179303"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -738,7 +759,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80180890"/>
+        <c:crossAx val="31763613"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -746,7 +767,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80180890"/>
+        <c:axId val="31763613"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -775,8 +796,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-GB" sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Youden Parameter (TPR-FPR)</a:t>
                 </a:r>
@@ -818,7 +843,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72898365"/>
+        <c:crossAx val="96179303"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -881,9 +906,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -1093,14 +1120,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>702360</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>114840</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>137880</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>6120</xdr:rowOff>
+      <xdr:colOff>136800</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>5040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1109,7 +1136,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="1515240" y="3323520"/>
-        <a:ext cx="5754240" cy="3792600"/>
+        <a:ext cx="5753160" cy="3791520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1233,7 +1260,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.99"/>
@@ -1508,7 +1535,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
         <v>24</v>
       </c>
@@ -1592,27 +1619,27 @@
         <v>31</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.31</v>
+        <v>0.39</v>
       </c>
       <c r="E16" s="6" t="n">
         <f aca="false">C16-D16</f>
-        <v>0.57</v>
+        <v>0.53</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>0.23</v>
       </c>
       <c r="H16" s="6" t="n">
         <f aca="false">F16-G16</f>
-        <v>0.65</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>32</v>
       </c>
@@ -1620,51 +1647,128 @@
         <v>33</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.34</v>
+        <v>0.31</v>
       </c>
       <c r="E17" s="6" t="n">
         <f aca="false">C17-D17</f>
-        <v>0.55</v>
+        <v>0.57</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="H17" s="6" t="n">
         <f aca="false">F17-G17</f>
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <f aca="false">C18-D18</f>
+        <v>0.55</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <f aca="false">F18-G18</f>
         <v>0.64</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="7" t="n">
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <f aca="false">C19-D19</f>
+        <v>0.63</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <f aca="false">F19-G19</f>
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.94</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <f aca="false">C20-D20</f>
+        <v>0.44</v>
+      </c>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="7" t="n">
         <v>0.67</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D21" s="7" t="n">
         <v>0.21</v>
       </c>
-      <c r="E18" s="7" t="n">
-        <f aca="false">C18-D18</f>
+      <c r="E21" s="7" t="n">
+        <f aca="false">C21-D21</f>
         <v>0.46</v>
       </c>
-      <c r="F18" s="7" t="n">
+      <c r="F21" s="7" t="n">
         <v>0.67</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G21" s="7" t="n">
         <v>0.21</v>
       </c>
-      <c r="H18" s="7" t="n">
-        <f aca="false">F18-G18</f>
+      <c r="H21" s="7" t="n">
+        <f aca="false">F21-G21</f>
         <v>0.46</v>
       </c>
     </row>

</xml_diff>